<commit_message>
rtmtools 0.6.1: fixes found by running the whole route on Mongolia's public aggregates
- rtmsample draw: a reserve larger than the units left after the selection is capped with a note
  (it still stops when n alone exceeds the units)
- rtminput, sampling: without a household list, the listing forms for the selected areas are
  written after the first stage (rtmlist prepare; new Design key segment_size, default 150) and
  the selected areas saved with their segments; a returned listing is checked against them
- rtminput: the area id's type is matched after rtmlist import before the merge
- rtminput: the phone sample is drawn among the households the Files sheet's phone column marks;
  a PSU with fewer owners than phone_per_psu is taken in full and the summary says how many
- exports record version 0.6.1; template and help carry segment_size
- tests/test_input.do: phone-sample assertions for the new rule; suite 13/13 pass

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/portable_do_files/rtm_inputs.xlsx
+++ b/portable_do_files/rtm_inputs.xlsx
@@ -902,7 +902,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D54"/>
+  <dimension ref="A1:D55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1556,441 +1556,463 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="3" t="inlineStr">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>segment_size</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Above how many households should a selected area be listed in segments (one segment chosen per area)?</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>default when blank: 150. households per listing segment: areas above it are listed in segments, one chosen at random per area (UN 2008 paras 138-140; 150 is a common field value)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
         <is>
           <t># phone subsample of a baseline (rtmsample draw, reserve all)</t>
         </is>
       </c>
-      <c r="C33" s="3" t="inlineStr">
+      <c r="C34" s="3" t="inlineStr">
         <is>
           <t>phone subsample of a baseline (rtmsample draw, reserve all)</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
+    <row r="35">
+      <c r="A35" t="inlineStr">
         <is>
           <t>phone_per_psu</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr">
+      <c r="B35" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
+      <c r="C35" t="inlineStr">
         <is>
           <t>How many households per PSU are called first (blank = no phone subsample; needs a baseline on Files)?</t>
         </is>
       </c>
-      <c r="D34" s="2" t="inlineStr">
+      <c r="D35" s="2" t="inlineStr">
         <is>
           <t>blank = not used. households per PSU called first, every other household an ordered replacement; blank = none (needs a baseline row in Files)</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="3" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
         <is>
           <t># random digit dialing (rtmsample rdd)</t>
         </is>
       </c>
-      <c r="C35" s="3" t="inlineStr">
+      <c r="C36" s="3" t="inlineStr">
         <is>
           <t>random digit dialing (rtmsample rdd)</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
+    <row r="37">
+      <c r="A37" t="inlineStr">
         <is>
           <t>rdd</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr">
+      <c r="B37" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr">
+      <c r="C37" t="inlineStr">
         <is>
           <t>Should phone numbers be generated from operator prefixes (random digit dialing)?</t>
         </is>
       </c>
-      <c r="D36" s="2" t="inlineStr">
+      <c r="D37" s="2" t="inlineStr">
         <is>
           <t>default when blank: no. yes | no: draw numbers from the Prefixes sheet; the numbers are never exported</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="3" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="3" t="inlineStr">
         <is>
           <t># weights of a round (rtmweight base, nonresponse, trim, calibrate, report)</t>
         </is>
       </c>
-      <c r="C37" s="3" t="inlineStr">
+      <c r="C38" s="3" t="inlineStr">
         <is>
           <t>weights of a round (rtmweight base, nonresponse, trim, calibrate, report)</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>base_weight</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>baseline</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>Where does the base weight come from?</t>
-        </is>
-      </c>
-      <c r="D38" s="2" t="inlineStr">
-        <is>
-          <t>default when blank: baseline. baseline | probabilities: the baseline weight redistributed to the phone sample, or 1 / product of the probabilities (HFPS Vol. 2 pp. 10-11, 21)</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>nonresponse</t>
+          <t>base_weight</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>propensity</t>
+          <t>baseline</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>How should the weights be adjusted for households not interviewed?</t>
+          <t>Where does the base weight come from?</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>default when blank: propensity. propensity | probit | classes | ebalance | ebalance_nobase | post | none (HFPS Vol. 2 Annex A2.3.1: propensity in deciles; ebalance and post are L2 program practice)</t>
+          <t>default when blank: baseline. baseline | probabilities: the baseline weight redistributed to the phone sample, or 1 / product of the probabilities (HFPS Vol. 2 pp. 10-11, 21)</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>covariates</t>
+          <t>nonresponse</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>urban i.educ head_age assets hhsize</t>
+          <t>propensity</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Which baseline variables predict response (for propensity or balancing; i. before a category variable)?</t>
+          <t>How should the weights be adjusted for households not interviewed?</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>blank = not used. baseline variables of the propensity model or of the balancing (i. for categories)</t>
+          <t>default when blank: propensity. propensity | probit | classes | ebalance | ebalance_nobase | post | none (HFPS Vol. 2 Annex A2.3.1: propensity in deciles; ebalance and post are L2 program practice)</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>classes</t>
+          <t>covariates</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>region urban</t>
+          <t>urban i.educ head_age assets hhsize</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Which variables define the weighting classes (for classes)?</t>
+          <t>Which baseline variables predict response (for propensity or balancing; i. before a category variable)?</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>blank = not used. class variables for nonresponse classes (UN 2008 section 6.5)</t>
+          <t>blank = not used. baseline variables of the propensity model or of the balancing (i. for categories)</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>cells</t>
+          <t>classes</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>region urban head_female agegrp</t>
+          <t>region urban</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Which Cells sheet columns define the cells (for post)?</t>
+          <t>Which variables define the weighting classes (for classes)?</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>blank = not used. cell variables for nonresponse post: the columns of the Cells sheet before total</t>
+          <t>blank = not used. class variables for nonresponse classes (UN 2008 section 6.5)</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>ngroups</t>
+          <t>cells</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>region urban head_female agegrp</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>How many propensity groups (10 = deciles)?</t>
+          <t>Which Cells sheet columns define the cells (for post)?</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>default when blank: 10 (command). propensity groups (deciles)</t>
+          <t>blank = not used. cell variables for nonresponse post: the columns of the Cells sheet before total</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>moments</t>
+          <t>ngroups</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>10</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Balance means only (1), also variances (2), also skewness (3)?</t>
+          <t>How many propensity groups (10 = deciles)?</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>default when blank: 1 (command). balancing moments: 1 means, 2 adds variances, 3 adds skewness</t>
+          <t>default when blank: 10 (command). propensity groups (deciles)</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>trim</t>
+          <t>moments</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Should extreme weights be trimmed?</t>
+          <t>Balance means only (1), also variances (2), also skewness (3)?</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>default when blank: none. none | winsor | cap (HFPS Vol. 2 p. 11 winsorises at the 98th percentile; UN 2008 section 6.8)</t>
+          <t>default when blank: 1 (command). balancing moments: 1 means, 2 adds variances, 3 adds skewness</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>trim_pct</t>
+          <t>trim</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>98</t>
+          <t>none</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>If winsor: at which percentile?</t>
+          <t>Should extreme weights be trimmed?</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>default when blank: 98 (command). winsorising percentile</t>
+          <t>default when blank: none. none | winsor | cap (HFPS Vol. 2 p. 11 winsorises at the 98th percentile; UN 2008 section 6.8)</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>trim_cap</t>
+          <t>trim_pct</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>98</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>If cap: at which value?</t>
+          <t>If winsor: at which percentile?</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>blank = not used. absolute cap for trim cap, or blank</t>
+          <t>default when blank: 98 (command). winsorising percentile</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>trim_capmult</t>
+          <t>trim_cap</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>If cap: at how many times the median?</t>
+          <t>If cap: at which value?</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>blank = not used. cap as a multiple of the median, or blank</t>
+          <t>blank = not used. absolute cap for trim cap, or blank</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>calibrate</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>rake</t>
+          <t>trim_capmult</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Should the weights be calibrated to the Totals sheet?</t>
+          <t>If cap: at how many times the median?</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>default when blank: none. none | rake | regress | post (Deville and Sarndal 1992; Deville, Sarndal and Sautory 1993)</t>
+          <t>blank = not used. cap as a multiple of the median, or blank</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>cal_vars</t>
+          <t>calibrate</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>region urban</t>
+          <t>rake</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Which variables to calibrate on (blank = every variable on Totals)?</t>
+          <t>Should the weights be calibrated to the Totals sheet?</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>blank = not used. categorical variables to calibrate on; every category must be on the Totals sheet; blank = every variable there</t>
+          <t>default when blank: none. none | rake | regress | post (Deville and Sarndal 1992; Deville, Sarndal and Sautory 1993)</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>cal_ll</t>
+          <t>cal_vars</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>region urban</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Lower bound on the calibration ratio (regress), or blank?</t>
+          <t>Which variables to calibrate on (blank = every variable on Totals)?</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>blank = not used. lower bound on the weight ratio (regress), or blank</t>
+          <t>blank = not used. categorical variables to calibrate on; every category must be on the Totals sheet; blank = every variable there</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>cal_ul</t>
+          <t>cal_ll</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Upper bound, or blank?</t>
+          <t>Lower bound on the calibration ratio (regress), or blank?</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>blank = not used. upper bound, or blank</t>
+          <t>blank = not used. lower bound on the weight ratio (regress), or blank</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>report_by</t>
-        </is>
-      </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>region</t>
+          <t>cal_ul</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Which variable should the report break the weights down by (blank = none)?</t>
+          <t>Upper bound, or blank?</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>blank = not used. variable for the by-group table of the weighting report, or blank</t>
+          <t>blank = not used. upper bound, or blank</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
+          <t>report_by</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>region</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Which variable should the report break the weights down by (blank = none)?</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>blank = not used. variable for the by-group table of the weighting report, or blank</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
           <t>report_files</t>
         </is>
       </c>
-      <c r="B54" t="inlineStr">
+      <c r="B55" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="C54" t="inlineStr">
+      <c r="C55" t="inlineStr">
         <is>
           <t>Write the Word method note and the Excel report?</t>
         </is>
       </c>
-      <c r="D54" s="2" t="inlineStr">
+      <c r="D55" s="2" t="inlineStr">
         <is>
           <t>default when blank: yes. yes | no: write the Word method note and the Excel report into output_dir</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="37">
+  <dataValidations count="38">
     <dataValidation sqref="B4" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Not a number" error="This row needs a number (or blank for the default)" promptTitle="seed" prompt="Which seed should every draw use (any whole number; keep it to repeat the draw)?" type="decimal" operator="greaterThanOrEqual">
       <formula1>-1000000000</formula1>
     </dataValidation>
@@ -2060,46 +2082,49 @@
     <dataValidation sqref="B32" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Not a number" error="This row needs a number (or blank for the default)" promptTitle="households_per_area" prompt="How many households per selected area (blank = none; needs a household list or listing on Files)?" type="decimal" operator="greaterThanOrEqual">
       <formula1>-1000000000</formula1>
     </dataValidation>
-    <dataValidation sqref="B34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Not a number" error="This row needs a number (or blank for the default)" promptTitle="phone_per_psu" prompt="How many households per PSU are called first (blank = no phone subsample; needs a baseline on Files)?" type="decimal" operator="greaterThanOrEqual">
+    <dataValidation sqref="B33" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Not a number" error="This row needs a number (or blank for the default)" promptTitle="segment_size" prompt="Above how many households should a selected area be listed in segments (one segment chosen per area)?" type="decimal" operator="greaterThanOrEqual">
       <formula1>-1000000000</formula1>
     </dataValidation>
-    <dataValidation sqref="B36" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Not an allowed value" error="Choose one of: yes, no (or leave blank for the default)" promptTitle="rdd" prompt="Should phone numbers be generated from operator prefixes (random digit dialing)?" type="list">
+    <dataValidation sqref="B35" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Not a number" error="This row needs a number (or blank for the default)" promptTitle="phone_per_psu" prompt="How many households per PSU are called first (blank = no phone subsample; needs a baseline on Files)?" type="decimal" operator="greaterThanOrEqual">
+      <formula1>-1000000000</formula1>
+    </dataValidation>
+    <dataValidation sqref="B37" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Not an allowed value" error="Choose one of: yes, no (or leave blank for the default)" promptTitle="rdd" prompt="Should phone numbers be generated from operator prefixes (random digit dialing)?" type="list">
       <formula1>"yes,no"</formula1>
     </dataValidation>
-    <dataValidation sqref="B38" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Not an allowed value" error="Choose one of: baseline, probabilities (or leave blank for the default)" promptTitle="base_weight" prompt="Where does the base weight come from?" type="list">
+    <dataValidation sqref="B39" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Not an allowed value" error="Choose one of: baseline, probabilities (or leave blank for the default)" promptTitle="base_weight" prompt="Where does the base weight come from?" type="list">
       <formula1>"baseline,probabilities"</formula1>
     </dataValidation>
-    <dataValidation sqref="B39" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Not an allowed value" error="Choose one of: propensity, probit, classes, ebalance, ebalance_nobase, post, none (or leave blank for the default)" promptTitle="nonresponse" prompt="How should the weights be adjusted for households not interviewed?" type="list">
+    <dataValidation sqref="B40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Not an allowed value" error="Choose one of: propensity, probit, classes, ebalance, ebalance_nobase, post, none (or leave blank for the default)" promptTitle="nonresponse" prompt="How should the weights be adjusted for households not interviewed?" type="list">
       <formula1>"propensity,probit,classes,ebalance,ebalance_nobase,post,none"</formula1>
     </dataValidation>
-    <dataValidation sqref="B43" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Not a number" error="This row needs a number (or blank for the default)" promptTitle="ngroups" prompt="How many propensity groups (10 = deciles)?" type="decimal" operator="greaterThanOrEqual">
+    <dataValidation sqref="B44" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Not a number" error="This row needs a number (or blank for the default)" promptTitle="ngroups" prompt="How many propensity groups (10 = deciles)?" type="decimal" operator="greaterThanOrEqual">
       <formula1>-1000000000</formula1>
     </dataValidation>
-    <dataValidation sqref="B44" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Not a number" error="This row needs a number (or blank for the default)" promptTitle="moments" prompt="Balance means only (1), also variances (2), also skewness (3)?" type="decimal" operator="greaterThanOrEqual">
+    <dataValidation sqref="B45" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Not a number" error="This row needs a number (or blank for the default)" promptTitle="moments" prompt="Balance means only (1), also variances (2), also skewness (3)?" type="decimal" operator="greaterThanOrEqual">
       <formula1>-1000000000</formula1>
     </dataValidation>
-    <dataValidation sqref="B45" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Not an allowed value" error="Choose one of: none, winsor, cap (or leave blank for the default)" promptTitle="trim" prompt="Should extreme weights be trimmed?" type="list">
+    <dataValidation sqref="B46" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Not an allowed value" error="Choose one of: none, winsor, cap (or leave blank for the default)" promptTitle="trim" prompt="Should extreme weights be trimmed?" type="list">
       <formula1>"none,winsor,cap"</formula1>
     </dataValidation>
-    <dataValidation sqref="B46" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Not a number" error="This row needs a number (or blank for the default)" promptTitle="trim_pct" prompt="If winsor: at which percentile?" type="decimal" operator="greaterThanOrEqual">
+    <dataValidation sqref="B47" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Not a number" error="This row needs a number (or blank for the default)" promptTitle="trim_pct" prompt="If winsor: at which percentile?" type="decimal" operator="greaterThanOrEqual">
       <formula1>-1000000000</formula1>
     </dataValidation>
-    <dataValidation sqref="B47" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Not a number" error="This row needs a number (or blank for the default)" promptTitle="trim_cap" prompt="If cap: at which value?" type="decimal" operator="greaterThanOrEqual">
+    <dataValidation sqref="B48" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Not a number" error="This row needs a number (or blank for the default)" promptTitle="trim_cap" prompt="If cap: at which value?" type="decimal" operator="greaterThanOrEqual">
       <formula1>-1000000000</formula1>
     </dataValidation>
-    <dataValidation sqref="B48" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Not a number" error="This row needs a number (or blank for the default)" promptTitle="trim_capmult" prompt="If cap: at how many times the median?" type="decimal" operator="greaterThanOrEqual">
+    <dataValidation sqref="B49" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Not a number" error="This row needs a number (or blank for the default)" promptTitle="trim_capmult" prompt="If cap: at how many times the median?" type="decimal" operator="greaterThanOrEqual">
       <formula1>-1000000000</formula1>
     </dataValidation>
-    <dataValidation sqref="B49" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Not an allowed value" error="Choose one of: none, rake, regress, post (or leave blank for the default)" promptTitle="calibrate" prompt="Should the weights be calibrated to the Totals sheet?" type="list">
+    <dataValidation sqref="B50" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Not an allowed value" error="Choose one of: none, rake, regress, post (or leave blank for the default)" promptTitle="calibrate" prompt="Should the weights be calibrated to the Totals sheet?" type="list">
       <formula1>"none,rake,regress,post"</formula1>
     </dataValidation>
-    <dataValidation sqref="B51" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Not a number" error="This row needs a number (or blank for the default)" promptTitle="cal_ll" prompt="Lower bound on the calibration ratio (regress), or blank?" type="decimal" operator="greaterThanOrEqual">
+    <dataValidation sqref="B52" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Not a number" error="This row needs a number (or blank for the default)" promptTitle="cal_ll" prompt="Lower bound on the calibration ratio (regress), or blank?" type="decimal" operator="greaterThanOrEqual">
       <formula1>-1000000000</formula1>
     </dataValidation>
-    <dataValidation sqref="B52" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Not a number" error="This row needs a number (or blank for the default)" promptTitle="cal_ul" prompt="Upper bound, or blank?" type="decimal" operator="greaterThanOrEqual">
+    <dataValidation sqref="B53" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Not a number" error="This row needs a number (or blank for the default)" promptTitle="cal_ul" prompt="Upper bound, or blank?" type="decimal" operator="greaterThanOrEqual">
       <formula1>-1000000000</formula1>
     </dataValidation>
-    <dataValidation sqref="B54" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Not an allowed value" error="Choose one of: yes, no (or leave blank for the default)" promptTitle="report_files" prompt="Write the Word method note and the Excel report?" type="list">
+    <dataValidation sqref="B55" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Not an allowed value" error="Choose one of: yes, no (or leave blank for the default)" promptTitle="report_files" prompt="Write the Word method note and the Excel report?" type="list">
       <formula1>"yes,no"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>